<commit_message>
Change api to expose (name, topic); Fix handling of excel files; add pack to watch command
</commit_message>
<xml_diff>
--- a/robots/src/rcc/readexcel/data/sample.xlsx
+++ b/robots/src/rcc/readexcel/data/sample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/moellenbeck/projects/atlasengine_contrib/reps/processcube-robot-agent/robots/src/rcc/readexcel/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D5275BF-FA88-1D43-9452-463079568A71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0254596-42EB-8748-86BC-B938F10A9E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="580" yWindow="740" windowWidth="28240" windowHeight="17160" xr2:uid="{08C3758B-374D-BC40-9E2F-7D4BDAC2F893}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Col 1</t>
   </si>
@@ -63,6 +63,12 @@
   </si>
   <si>
     <t>val 2.4</t>
+  </si>
+  <si>
+    <t>val 1.5</t>
+  </si>
+  <si>
+    <t>val 2.5</t>
   </si>
 </sst>
 </file>
@@ -414,7 +420,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D422F2C0-5A4E-0D48-BABB-BBD1552721FE}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -457,6 +463,14 @@
         <v>9</v>
       </c>
     </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>